<commit_message>
Add auto-deploy workflow and cache busting for data updates
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\명찰\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A498F48D-C98A-4455-8174-77E52117731B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BB23D5-BBD0-4040-9CEC-DA75388274AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19290" windowHeight="9540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="126">
   <si>
     <t xml:space="preserve">러닝센터 명찰제작 양식 </t>
     <phoneticPr fontId="4" type="noConversion"/>
@@ -326,6 +326,100 @@
     <t>25년 서비스센터 실장 
 데이터 역량 교육</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>선택 특강</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>3. 성과관리/ 피플 리더십</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. 데이터 핸들링 기초 역량 업그레이드</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>3. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>4. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>3. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>4. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>5. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>4. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>5. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>6. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>5. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>6. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>7. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>6. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>7. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>8. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>7. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>8. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>9. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>8. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>9. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>10. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>9. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>10. 데이터 핸들링 기초 역량 업그레이드</t>
+  </si>
+  <si>
+    <t>11. 성과관리/ 피플 리더십</t>
+  </si>
+  <si>
+    <t>10. AI Tool을 활용한 서비스 문제해결 워크샵</t>
+  </si>
+  <si>
+    <t>11. 데이터 핸들링 기초 역량 업그레이드</t>
   </si>
 </sst>
 </file>
@@ -1640,29 +1734,29 @@
     <xf numFmtId="0" fontId="6" fillId="36" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="238">
@@ -2239,51 +2333,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E53"/>
+  <dimension ref="A2:F53"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="15.77734375" customWidth="1"/>
+    <col min="3" max="6" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="20.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:6" ht="20.25">
+      <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5" ht="54" customHeight="1">
-      <c r="A3" s="6" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="54" customHeight="1">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4" spans="1:5" ht="16.5">
-      <c r="A4" s="6" t="s">
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+    </row>
+    <row r="4" spans="1:6" ht="16.5">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16.5" customHeight="1">
+    <row r="5" spans="1:6" ht="16.5" customHeight="1">
       <c r="A5" s="8" t="s">
         <v>6</v>
       </c>
@@ -2293,14 +2392,15 @@
       <c r="C5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D5" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="D5" s="2"/>
+      <c r="E5" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" customHeight="1">
+    <row r="6" spans="1:6" ht="16.5" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="1" t="s">
         <v>87</v>
@@ -2308,14 +2408,15 @@
       <c r="C6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="D6" s="2"/>
+      <c r="E6" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" customHeight="1">
+    <row r="7" spans="1:6" ht="16.5" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="1" t="s">
         <v>86</v>
@@ -2323,29 +2424,35 @@
       <c r="C7" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E7" s="10">
+      <c r="D7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F7" s="7">
         <v>318537</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5">
+    <row r="8" spans="1:6" ht="16.5">
       <c r="A8" s="8"/>
       <c r="B8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="D8" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1">
+    <row r="9" spans="1:6" ht="13.5" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>5</v>
       </c>
@@ -2355,14 +2462,17 @@
       <c r="C9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E9" s="1">
+      <c r="D9" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F9" s="1">
         <v>293575</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5">
+    <row r="10" spans="1:6" ht="16.5">
       <c r="A10" s="8"/>
       <c r="B10" s="1" t="s">
         <v>48</v>
@@ -2370,14 +2480,17 @@
       <c r="C10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E10" s="1">
+      <c r="D10" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F10" s="1">
         <v>294004</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="16.5">
+    <row r="11" spans="1:6" ht="16.5">
       <c r="A11" s="8"/>
       <c r="B11" s="1" t="s">
         <v>49</v>
@@ -2385,14 +2498,17 @@
       <c r="C11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E11" s="1">
+      <c r="D11" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F11" s="1">
         <v>292052</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="16.5">
+    <row r="12" spans="1:6" ht="16.5">
       <c r="A12" s="8"/>
       <c r="B12" s="1" t="s">
         <v>49</v>
@@ -2400,14 +2516,17 @@
       <c r="C12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E12" s="1">
+      <c r="D12" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F12" s="1">
         <v>292052</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="16.5">
+    <row r="13" spans="1:6" ht="16.5">
       <c r="A13" s="8"/>
       <c r="B13" s="1" t="s">
         <v>50</v>
@@ -2415,14 +2534,17 @@
       <c r="C13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E13" s="1">
+      <c r="D13" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F13" s="1">
         <v>293976</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="16.5">
+    <row r="14" spans="1:6" ht="16.5">
       <c r="A14" s="8"/>
       <c r="B14" s="1" t="s">
         <v>51</v>
@@ -2430,14 +2552,17 @@
       <c r="C14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E14" s="1">
+      <c r="D14" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F14" s="1">
         <v>289090</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="16.5">
+    <row r="15" spans="1:6" ht="16.5">
       <c r="A15" s="8"/>
       <c r="B15" s="1" t="s">
         <v>52</v>
@@ -2445,14 +2570,17 @@
       <c r="C15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E15" s="1">
+      <c r="D15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F15" s="1">
         <v>293378</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="16.5">
+    <row r="16" spans="1:6" ht="16.5">
       <c r="A16" s="8"/>
       <c r="B16" s="1" t="s">
         <v>53</v>
@@ -2460,14 +2588,17 @@
       <c r="C16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E16" s="1">
+      <c r="D16" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F16" s="1">
         <v>292659</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="16.5">
+    <row r="17" spans="1:6" ht="16.5">
       <c r="A17" s="8"/>
       <c r="B17" s="1" t="s">
         <v>54</v>
@@ -2475,14 +2606,17 @@
       <c r="C17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E17" s="1">
+      <c r="D17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F17" s="1">
         <v>292672</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="16.5">
+    <row r="18" spans="1:6" ht="16.5">
       <c r="A18" s="8"/>
       <c r="B18" s="1" t="s">
         <v>55</v>
@@ -2490,14 +2624,17 @@
       <c r="C18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E18" s="1">
+      <c r="D18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F18" s="1">
         <v>294269</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="16.5">
+    <row r="19" spans="1:6" ht="16.5">
       <c r="A19" s="8"/>
       <c r="B19" s="1" t="s">
         <v>56</v>
@@ -2505,14 +2642,17 @@
       <c r="C19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E19" s="1">
+      <c r="D19" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F19" s="1">
         <v>292325</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="16.5">
+    <row r="20" spans="1:6" ht="16.5">
       <c r="A20" s="8"/>
       <c r="B20" s="1" t="s">
         <v>57</v>
@@ -2520,14 +2660,17 @@
       <c r="C20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E20" s="1">
+      <c r="D20" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E20" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F20" s="1">
         <v>293533</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="16.5">
+    <row r="21" spans="1:6" ht="16.5">
       <c r="A21" s="8"/>
       <c r="B21" s="1" t="s">
         <v>58</v>
@@ -2535,14 +2678,17 @@
       <c r="C21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E21" s="1">
+      <c r="D21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E21" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F21" s="1">
         <v>291742</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="16.5">
+    <row r="22" spans="1:6" ht="16.5">
       <c r="A22" s="8"/>
       <c r="B22" s="1" t="s">
         <v>59</v>
@@ -2550,14 +2696,17 @@
       <c r="C22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E22" s="1">
+      <c r="D22" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F22" s="1">
         <v>293692</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="16.5">
+    <row r="23" spans="1:6" ht="16.5">
       <c r="A23" s="8"/>
       <c r="B23" s="1" t="s">
         <v>60</v>
@@ -2565,14 +2714,17 @@
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E23" s="1">
+      <c r="D23" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E23" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F23" s="1">
         <v>293127</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="16.5">
+    <row r="24" spans="1:6" ht="16.5">
       <c r="A24" s="8"/>
       <c r="B24" s="1" t="s">
         <v>61</v>
@@ -2580,14 +2732,17 @@
       <c r="C24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E24" s="1">
+      <c r="D24" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F24" s="1">
         <v>293979</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="16.5">
+    <row r="25" spans="1:6" ht="16.5">
       <c r="A25" s="8"/>
       <c r="B25" s="1" t="s">
         <v>62</v>
@@ -2595,14 +2750,17 @@
       <c r="C25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E25" s="1">
+      <c r="D25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F25" s="1">
         <v>292961</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="16.5">
+    <row r="26" spans="1:6" ht="16.5">
       <c r="A26" s="8"/>
       <c r="B26" s="1" t="s">
         <v>63</v>
@@ -2610,14 +2768,17 @@
       <c r="C26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E26" s="1">
+      <c r="D26" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E26" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F26" s="1">
         <v>293130</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="16.5">
+    <row r="27" spans="1:6" ht="16.5">
       <c r="A27" s="8"/>
       <c r="B27" s="1" t="s">
         <v>64</v>
@@ -2625,14 +2786,17 @@
       <c r="C27" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E27" s="1">
+      <c r="D27" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F27" s="1">
         <v>292917</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="16.5">
+    <row r="28" spans="1:6" ht="16.5">
       <c r="A28" s="8"/>
       <c r="B28" s="1" t="s">
         <v>65</v>
@@ -2640,14 +2804,17 @@
       <c r="C28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E28" s="1">
+      <c r="D28" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E28" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F28" s="1">
         <v>294351</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="16.5">
+    <row r="29" spans="1:6" ht="16.5">
       <c r="A29" s="8"/>
       <c r="B29" s="1" t="s">
         <v>66</v>
@@ -2655,14 +2822,17 @@
       <c r="C29" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E29" s="1">
+      <c r="D29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E29" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F29" s="1">
         <v>294306</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="16.5">
+    <row r="30" spans="1:6" ht="16.5">
       <c r="A30" s="8"/>
       <c r="B30" s="1" t="s">
         <v>61</v>
@@ -2670,14 +2840,17 @@
       <c r="C30" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E30" s="1">
+      <c r="D30" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E30" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F30" s="1">
         <v>293131</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="16.5">
+    <row r="31" spans="1:6" ht="16.5">
       <c r="A31" s="8"/>
       <c r="B31" s="1" t="s">
         <v>67</v>
@@ -2685,14 +2858,17 @@
       <c r="C31" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D31" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E31" s="1">
+      <c r="D31" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E31" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F31" s="1">
         <v>292371</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="16.5">
+    <row r="32" spans="1:6" ht="16.5">
       <c r="A32" s="8"/>
       <c r="B32" s="1" t="s">
         <v>68</v>
@@ -2700,14 +2876,17 @@
       <c r="C32" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D32" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E32" s="1">
+      <c r="D32" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E32" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F32" s="1">
         <v>294307</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="16.5">
+    <row r="33" spans="1:6" ht="16.5">
       <c r="A33" s="8"/>
       <c r="B33" s="1" t="s">
         <v>69</v>
@@ -2715,14 +2894,17 @@
       <c r="C33" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E33" s="1">
+      <c r="D33" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E33" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F33" s="1">
         <v>293134</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="16.5">
+    <row r="34" spans="1:6" ht="16.5">
       <c r="A34" s="8"/>
       <c r="B34" s="1" t="s">
         <v>70</v>
@@ -2730,14 +2912,17 @@
       <c r="C34" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D34" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E34" s="1">
+      <c r="D34" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E34" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F34" s="1">
         <v>293007</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="16.5">
+    <row r="35" spans="1:6" ht="16.5">
       <c r="A35" s="8"/>
       <c r="B35" s="1" t="s">
         <v>71</v>
@@ -2745,14 +2930,17 @@
       <c r="C35" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D35" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E35" s="1">
+      <c r="D35" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E35" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F35" s="1">
         <v>292202</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="16.5">
+    <row r="36" spans="1:6" ht="16.5">
       <c r="A36" s="8"/>
       <c r="B36" s="1" t="s">
         <v>72</v>
@@ -2760,14 +2948,17 @@
       <c r="C36" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D36" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E36" s="1">
+      <c r="D36" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E36" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F36" s="1">
         <v>292763</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="16.5">
+    <row r="37" spans="1:6" ht="16.5">
       <c r="A37" s="8"/>
       <c r="B37" s="1" t="s">
         <v>73</v>
@@ -2775,14 +2966,17 @@
       <c r="C37" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D37" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E37" s="1">
+      <c r="D37" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E37" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F37" s="1">
         <v>293262</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="16.5">
+    <row r="38" spans="1:6" ht="16.5">
       <c r="A38" s="8"/>
       <c r="B38" s="1" t="s">
         <v>74</v>
@@ -2790,14 +2984,17 @@
       <c r="C38" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D38" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E38" s="1">
+      <c r="D38" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F38" s="1">
         <v>293287</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="16.5">
+    <row r="39" spans="1:6" ht="16.5">
       <c r="A39" s="8"/>
       <c r="B39" s="1" t="s">
         <v>75</v>
@@ -2805,14 +3002,17 @@
       <c r="C39" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D39" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E39" s="1">
+      <c r="D39" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E39" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F39" s="1">
         <v>293463</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="16.5">
+    <row r="40" spans="1:6" ht="16.5">
       <c r="A40" s="8"/>
       <c r="B40" s="1" t="s">
         <v>76</v>
@@ -2820,14 +3020,17 @@
       <c r="C40" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D40" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E40" s="1">
+      <c r="D40" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E40" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F40" s="1">
         <v>289000</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="16.5">
+    <row r="41" spans="1:6" ht="16.5">
       <c r="A41" s="8"/>
       <c r="B41" s="1" t="s">
         <v>75</v>
@@ -2835,14 +3038,17 @@
       <c r="C41" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D41" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E41" s="1">
+      <c r="D41" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F41" s="1">
         <v>293464</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="16.5">
+    <row r="42" spans="1:6" ht="16.5">
       <c r="A42" s="8"/>
       <c r="B42" s="1" t="s">
         <v>77</v>
@@ -2850,14 +3056,17 @@
       <c r="C42" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D42" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E42" s="1">
+      <c r="D42" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E42" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F42" s="1">
         <v>292789</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="16.5">
+    <row r="43" spans="1:6" ht="16.5">
       <c r="A43" s="8"/>
       <c r="B43" s="1" t="s">
         <v>78</v>
@@ -2865,14 +3074,17 @@
       <c r="C43" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D43" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E43" s="1">
+      <c r="D43" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E43" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F43" s="1">
         <v>293434</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="16.5">
+    <row r="44" spans="1:6" ht="16.5">
       <c r="A44" s="8"/>
       <c r="B44" s="1" t="s">
         <v>79</v>
@@ -2880,14 +3092,17 @@
       <c r="C44" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D44" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E44" s="1">
+      <c r="D44" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E44" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F44" s="1">
         <v>292610</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="16.5">
+    <row r="45" spans="1:6" ht="16.5">
       <c r="A45" s="8"/>
       <c r="B45" s="1" t="s">
         <v>80</v>
@@ -2895,14 +3110,17 @@
       <c r="C45" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D45" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E45" s="1">
+      <c r="D45" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E45" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F45" s="1">
         <v>294322</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="16.5">
+    <row r="46" spans="1:6" ht="16.5">
       <c r="A46" s="8"/>
       <c r="B46" s="1" t="s">
         <v>81</v>
@@ -2910,14 +3128,17 @@
       <c r="C46" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D46" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E46" s="1">
+      <c r="D46" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E46" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F46" s="1">
         <v>293962</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="16.5">
+    <row r="47" spans="1:6" ht="16.5">
       <c r="A47" s="8"/>
       <c r="B47" s="1" t="s">
         <v>60</v>
@@ -2925,14 +3146,17 @@
       <c r="C47" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D47" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E47" s="1">
+      <c r="D47" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E47" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F47" s="1">
         <v>293442</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="16.5">
+    <row r="48" spans="1:6" ht="16.5">
       <c r="A48" s="8"/>
       <c r="B48" s="1" t="s">
         <v>82</v>
@@ -2940,14 +3164,17 @@
       <c r="C48" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D48" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E48" s="1">
+      <c r="D48" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E48" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F48" s="1">
         <v>292802</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="16.5">
+    <row r="49" spans="1:6" ht="16.5">
       <c r="A49" s="8"/>
       <c r="B49" s="3" t="s">
         <v>91</v>
@@ -2955,40 +3182,55 @@
       <c r="C49" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D49" s="9">
-        <v>45946</v>
-      </c>
-      <c r="E49" s="3">
+      <c r="D49" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E49" s="6">
+        <v>45946</v>
+      </c>
+      <c r="F49" s="3">
         <v>292091</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="16.5">
+    <row r="50" spans="1:6" ht="16.5">
       <c r="A50" s="8"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="1"/>
-    </row>
-    <row r="51" spans="1:5" ht="16.5">
+      <c r="D50" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E50" s="6"/>
+      <c r="F50" s="1"/>
+    </row>
+    <row r="51" spans="1:6" ht="16.5">
       <c r="A51" s="8"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="1"/>
-    </row>
-    <row r="52" spans="1:5" ht="16.5">
+      <c r="D51" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E51" s="6"/>
+      <c r="F51" s="1"/>
+    </row>
+    <row r="52" spans="1:6" ht="16.5">
       <c r="A52" s="8"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="1"/>
-    </row>
-    <row r="53" spans="1:5" ht="16.5">
+      <c r="D52" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E52" s="6"/>
+      <c r="F52" s="1"/>
+    </row>
+    <row r="53" spans="1:6" ht="16.5">
       <c r="A53" s="8"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="1"/>
+      <c r="D53" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" s="1"/>
     </row>
   </sheetData>
   <sortState ref="B8:C51">
@@ -2997,8 +3239,8 @@
   <mergeCells count="4">
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="A9:A53"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B3:F3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>